<commit_message>
update excel file 24.03.25
</commit_message>
<xml_diff>
--- a/URS_Certifications 19.03.25.xlsx
+++ b/URS_Certifications 19.03.25.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\сайт\сайт2\Сайт на практику\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25E4E60-6417-4AA1-92B7-46E869921B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA0FD9EC-DB3A-40EE-9D90-818A5DDFDCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet name="URS_Certifications (69)" sheetId="1" r:id="rId1"/>
+    <sheet name="URS_Certifications (70)" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5851" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5861" uniqueCount="714">
   <si>
     <t>Название компании</t>
   </si>
@@ -2167,7 +2167,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3028,16 +3028,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1310"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G1312"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="8.88671875" style="1"/>
-    <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="1"/>
-    <col min="7" max="7" width="13.44140625" style="1" customWidth="1"/>
+    <col min="1" max="6" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="10.5546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -29924,33 +29920,48 @@
       <c r="F1307" s="1" t="s">
         <v>326</v>
       </c>
+      <c r="G1307" s="2">
+        <v>46823</v>
+      </c>
     </row>
     <row r="1308" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1308" s="1" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B1308" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1308" s="1">
-        <v>6230126270</v>
+        <v>712</v>
+      </c>
+      <c r="D1308" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="E1308" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="F1308" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G1308" s="2">
+        <v>46824</v>
       </c>
     </row>
     <row r="1309" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1309" s="1" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B1309" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1309" s="1">
-        <v>6230126270</v>
+        <v>712</v>
+      </c>
+      <c r="D1309" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="E1309" s="1" t="s">
-        <v>710</v>
+        <v>26</v>
+      </c>
+      <c r="F1309" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G1309" s="2">
+        <v>46824</v>
       </c>
     </row>
     <row r="1310" spans="1:7" x14ac:dyDescent="0.3">
@@ -29964,6 +29975,34 @@
         <v>6230126270</v>
       </c>
       <c r="E1310" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1311" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1311" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1311" s="1">
+        <v>6230126270</v>
+      </c>
+      <c r="E1311" s="1" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1312" s="1" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1312" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1312" s="1">
+        <v>6230126270</v>
+      </c>
+      <c r="E1312" s="1" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>